<commit_message>
fixing vulnerability in .gitignore
</commit_message>
<xml_diff>
--- a/docs/22_Validation_Results.xlsx
+++ b/docs/22_Validation_Results.xlsx
@@ -135,7 +135,7 @@
     <t>STARTING A NEW RUN</t>
   </si>
   <si>
-    <t>Doc 21 Phase 6 requires the suite to be re-run after any fact-table reload. Eleven of the seventeen are data-dependent — the Check Catalog tab marks which. Re-run all seventeen anyway unless you are short of time; the six structural checks cost minutes.</t>
+    <t>Doc 21 Phase 6 requires the suite to be re-run after any fact-table reload. Twelve of the seventeen are data-dependent — the Check Catalog tab marks which. Re-run all seventeen anyway unless you are short of time; the five structural checks cost minutes.</t>
   </si>
   <si>
     <t>On Check Results, select the seventeen rows of the most recent run and copy them.</t>
@@ -345,7 +345,7 @@
     <t>Referential integrity</t>
   </si>
   <si>
-    <t>The §6.4 coverage query returns zero rows</t>
+    <t>The §6.5 coverage query returns zero rows</t>
   </si>
   <si>
     <t>Date relationship integrity</t>
@@ -456,7 +456,7 @@
     <t>SSMS or Power BI</t>
   </si>
   <si>
-    <t>Group FactSectorSales by DateKey for category 44X72 and confirm one row per month from pStartPeriod to pEndPeriod. A COUNTROWS card by year is enough.</t>
+    <t>Group FactSectorSales by DateKey for category 44X72 and confirm one row per month from pStartPeriod through the latest published MARTS month. A COUNTROWS card by year is enough.</t>
   </si>
   <si>
     <t>Treating an overlapping category set as a partition, and reporting a sum that double-counts.</t>
@@ -480,7 +480,7 @@
     <t>Unmapped category or item-type codes, which appear in the reports as a blank slicer entry.</t>
   </si>
   <si>
-    <t>Run the coverage query in doc 02 §6.4. A non-zero result lists exactly which codes are missing from RefMappings.xlsx.</t>
+    <t>Run the coverage query in doc 02 §6.5. A non-zero result lists exactly which codes are missing from RefMappings.xlsx.</t>
   </si>
   <si>
     <t>Fact dates outside the DimDate range. Power BI creates a blank row silently and time intelligence goes quietly wrong.</t>

</xml_diff>

<commit_message>
final edits to flawed M code for first API JSON data source
</commit_message>
<xml_diff>
--- a/docs/22_Validation_Results.xlsx
+++ b/docs/22_Validation_Results.xlsx
@@ -1424,7 +1424,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="42" customHeight="1" s="42">
+    <row r="55" ht="56.5" customHeight="1" s="42">
       <c r="B55" s="1" t="inlineStr">
         <is>
           <t>docs/validation/</t>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>One step-by-step procedure per check, V01 to V17, written for someone who has never run it. Each exists as a .docx to read and an .xlsx with a Pass/Fail drop-down on every step. The results still belong here, on Check Results — the V files are the instructions, not the record.</t>
+          <t>One step-by-step procedure per check, V01 to V17, written for someone who has never run it. Each exists as a .docx to read and an .xlsx with a Pass/Fail drop-down on every tick table (V07, V08, V15, V16 and V17). The results still belong here, on Check Results — the V files are the instructions, not the record.</t>
         </is>
       </c>
     </row>
@@ -2184,6 +2184,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1" s="42">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -4346,6 +4347,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1" s="42">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -12612,6 +12614,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1" s="42">
       <c r="A4" s="8" t="inlineStr">
         <is>
@@ -13487,6 +13490,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="34" customHeight="1" s="42">
       <c r="A4" s="8" t="inlineStr">
         <is>

</xml_diff>